<commit_message>
Add Chile presidency recipe
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P103"/>
+  <dimension ref="A1:P104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,6 @@
           <t>Afghanistan</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>4</v>
       </c>
@@ -533,17 +532,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -561,7 +554,6 @@
           <t>Albania</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>8</v>
       </c>
@@ -585,17 +577,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -613,7 +599,6 @@
           <t>Armenia</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>51</v>
       </c>
@@ -637,17 +622,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -665,7 +644,6 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>36</v>
       </c>
@@ -689,17 +667,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -717,7 +689,6 @@
           <t>Austria</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>40</v>
       </c>
@@ -741,17 +712,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -769,7 +734,6 @@
           <t>Azerbaijan</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>31</v>
       </c>
@@ -793,17 +757,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -821,7 +779,6 @@
           <t>Bangladesh</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>50</v>
       </c>
@@ -845,17 +802,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -873,7 +824,6 @@
           <t>Belarus</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>112</v>
       </c>
@@ -897,17 +847,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -925,7 +869,6 @@
           <t>Belgium</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>56</v>
       </c>
@@ -949,17 +892,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -977,7 +914,6 @@
           <t>Bhutan</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>64</v>
       </c>
@@ -1001,17 +937,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1029,7 +959,6 @@
           <t>Bulgaria</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
         <v>100</v>
       </c>
@@ -1053,17 +982,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1081,7 +1004,6 @@
           <t>Burundi</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>108</v>
       </c>
@@ -1105,17 +1027,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1133,7 +1049,6 @@
           <t>Cameroon</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
         <v>120</v>
       </c>
@@ -1157,17 +1072,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1185,7 +1094,6 @@
           <t>Costa Rica</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="n">
         <v>188</v>
       </c>
@@ -1209,17 +1117,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1237,7 +1139,6 @@
           <t>Croatia</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
         <v>191</v>
       </c>
@@ -1261,17 +1162,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1289,7 +1184,6 @@
           <t>Cuba</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="n">
         <v>192</v>
       </c>
@@ -1313,17 +1207,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1341,7 +1229,6 @@
           <t>Cyprus</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
         <v>196</v>
       </c>
@@ -1365,17 +1252,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1393,7 +1274,6 @@
           <t>Czechia</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
         <v>203</v>
       </c>
@@ -1417,17 +1297,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1445,7 +1319,6 @@
           <t>Denmark</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="n">
         <v>208</v>
       </c>
@@ -1469,17 +1342,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -1502,7 +1369,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>atlanticcouncil.org</t>
@@ -1528,16 +1394,11 @@
           <t>Mohamed Morsi</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1560,7 +1421,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>bbc.com</t>
@@ -1586,16 +1446,11 @@
           <t>Hosni Mubarak</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1618,7 +1473,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>c-span.org</t>
@@ -1644,16 +1498,11 @@
           <t>Mohamed Morsi</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1676,7 +1525,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>cdm15795.contentdm.oclc.org</t>
@@ -1702,16 +1550,11 @@
           <t>Hosni Mubarak</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1734,7 +1577,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>ilsoncenter.org</t>
@@ -1760,16 +1602,11 @@
           <t>Mohamed Morsi</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1792,7 +1629,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>leftvoice.org</t>
@@ -1818,16 +1654,11 @@
           <t>Hosni Mubarak</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1850,7 +1681,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>sadat.umd.edu</t>
@@ -1876,16 +1706,11 @@
           <t>Sadat (old speeches)</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1908,7 +1733,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>sis.gov.eg</t>
@@ -1919,7 +1743,6 @@
           <t>http://sis.gov.eg</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -1930,16 +1753,11 @@
           <t>Pres Sisi</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -1962,7 +1780,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>theguardian.com</t>
@@ -1988,16 +1805,11 @@
           <t>Hosni Mubarak</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -2020,7 +1832,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>youtube.com</t>
@@ -2046,16 +1857,11 @@
           <t>Amadou Toumani Touré; Dioncounda Traoré ; Hosni Mubarak; Mahamadou Issoufou; Mohamed Morsi; Moncef Marzouki</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (6 link(s))</t>
@@ -2073,7 +1879,6 @@
           <t>Estonia</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="n">
         <v>233</v>
       </c>
@@ -2097,17 +1902,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2125,7 +1924,6 @@
           <t>Ethiopia</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="n">
         <v>231</v>
       </c>
@@ -2149,17 +1947,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2182,7 +1974,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>pmo.gov.et</t>
@@ -2208,16 +1999,11 @@
           <t>Prime Minister Abiy Ahmed</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (2 link(s))</t>
@@ -2235,7 +2021,6 @@
           <t>Fiji</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="n">
         <v>242</v>
       </c>
@@ -2259,17 +2044,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2287,7 +2066,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="n">
         <v>246</v>
       </c>
@@ -2311,17 +2089,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2339,7 +2111,6 @@
           <t>Gambia</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="n">
         <v>270</v>
       </c>
@@ -2363,17 +2134,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2391,7 +2156,6 @@
           <t>Georgia</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
         <v>268</v>
       </c>
@@ -2415,17 +2179,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2443,7 +2201,6 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="n">
         <v>276</v>
       </c>
@@ -2467,17 +2224,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2495,7 +2246,6 @@
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
         <v>288</v>
       </c>
@@ -2519,17 +2269,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2547,7 +2291,6 @@
           <t>Greece</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="n">
         <v>300</v>
       </c>
@@ -2571,17 +2314,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2599,7 +2336,6 @@
           <t>Guyana</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
         <v>328</v>
       </c>
@@ -2623,17 +2359,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2651,7 +2381,6 @@
           <t>Hungary</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
         <v>348</v>
       </c>
@@ -2675,17 +2404,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2703,7 +2426,6 @@
           <t>Iceland</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="n">
         <v>352</v>
       </c>
@@ -2727,17 +2449,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2755,7 +2471,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
         <v>356</v>
       </c>
@@ -2779,17 +2494,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2807,7 +2516,6 @@
           <t>Iran, Islamic Republic of</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
         <v>364</v>
       </c>
@@ -2831,17 +2539,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2859,7 +2561,6 @@
           <t>Ireland</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="n">
         <v>372</v>
       </c>
@@ -2883,17 +2584,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2911,7 +2606,6 @@
           <t>Israel</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="n">
         <v>376</v>
       </c>
@@ -2935,17 +2629,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -2963,7 +2651,6 @@
           <t>Italy</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="n">
         <v>380</v>
       </c>
@@ -2987,17 +2674,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3015,7 +2696,6 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
       <c r="D49" t="n">
         <v>392</v>
       </c>
@@ -3039,17 +2719,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3067,7 +2741,6 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
       <c r="D50" t="n">
         <v>400</v>
       </c>
@@ -3091,17 +2764,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3119,7 +2786,6 @@
           <t>Kazakhstan</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
       <c r="D51" t="n">
         <v>398</v>
       </c>
@@ -3143,17 +2809,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3171,7 +2831,6 @@
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
       <c r="D52" t="n">
         <v>404</v>
       </c>
@@ -3195,17 +2854,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3223,7 +2876,6 @@
           <t>Kuwait</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
       <c r="D53" t="n">
         <v>414</v>
       </c>
@@ -3247,17 +2899,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3275,7 +2921,6 @@
           <t>Kyrgyzstan</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
       <c r="D54" t="n">
         <v>417</v>
       </c>
@@ -3299,17 +2944,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3327,7 +2966,6 @@
           <t>Latvia</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
       <c r="D55" t="n">
         <v>428</v>
       </c>
@@ -3351,17 +2989,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3379,7 +3011,6 @@
           <t>Lebanon</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="n">
         <v>422</v>
       </c>
@@ -3403,17 +3034,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3431,7 +3056,6 @@
           <t>Lesotho</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="n">
         <v>426</v>
       </c>
@@ -3455,17 +3079,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3483,7 +3101,6 @@
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
       <c r="D58" t="n">
         <v>440</v>
       </c>
@@ -3507,17 +3124,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3535,7 +3146,6 @@
           <t>Luxembourg</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="n">
         <v>442</v>
       </c>
@@ -3559,17 +3169,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3587,7 +3191,6 @@
           <t>Madagascar</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
       <c r="D60" t="n">
         <v>450</v>
       </c>
@@ -3611,17 +3214,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3639,7 +3236,6 @@
           <t>Maldives</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
       <c r="D61" t="n">
         <v>462</v>
       </c>
@@ -3663,17 +3259,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3691,7 +3281,6 @@
           <t>Malta</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
       <c r="D62" t="n">
         <v>470</v>
       </c>
@@ -3715,17 +3304,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3743,7 +3326,6 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
       <c r="D63" t="n">
         <v>484</v>
       </c>
@@ -3767,17 +3349,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3795,7 +3371,6 @@
           <t>Moldova, Republic of</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
       <c r="D64" t="n">
         <v>498</v>
       </c>
@@ -3819,17 +3394,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3847,7 +3416,6 @@
           <t>Morocco</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
       <c r="D65" t="n">
         <v>504</v>
       </c>
@@ -3871,17 +3439,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3899,7 +3461,6 @@
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="n">
         <v>528</v>
       </c>
@@ -3923,17 +3484,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -3951,7 +3506,6 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
       <c r="D67" t="n">
         <v>554</v>
       </c>
@@ -3975,17 +3529,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4008,7 +3556,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
           <t>books.google.com</t>
@@ -4034,16 +3581,11 @@
           <t>Olusegun Obasanjo</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -4066,7 +3608,6 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
           <t>statehouse.gov.ng</t>
@@ -4092,16 +3633,11 @@
           <t>Bola Ahmed Tinubu</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
           <t>from LeadersSpeeches_Africa.xlsx (1 link(s))</t>
@@ -4119,7 +3655,6 @@
           <t>North Macedonia</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
         <v>807</v>
       </c>
@@ -4143,17 +3678,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4171,7 +3700,6 @@
           <t>Norway</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="n">
         <v>578</v>
       </c>
@@ -4195,17 +3723,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4223,7 +3745,6 @@
           <t>Poland</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
       <c r="D72" t="n">
         <v>616</v>
       </c>
@@ -4247,17 +3768,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4275,7 +3790,6 @@
           <t>Romania</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="n">
         <v>642</v>
       </c>
@@ -4299,17 +3813,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4327,7 +3835,6 @@
           <t>Serbia</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="n">
         <v>688</v>
       </c>
@@ -4351,17 +3858,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4379,7 +3880,6 @@
           <t>Seychelles</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="n">
         <v>690</v>
       </c>
@@ -4403,17 +3903,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4431,7 +3925,6 @@
           <t>Sierra Leone</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
       <c r="D76" t="n">
         <v>694</v>
       </c>
@@ -4455,17 +3948,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4483,7 +3970,6 @@
           <t>Singapore</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
         <v>702</v>
       </c>
@@ -4507,17 +3993,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4535,7 +4015,6 @@
           <t>Slovakia</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
       <c r="D78" t="n">
         <v>703</v>
       </c>
@@ -4559,17 +4038,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4587,7 +4060,6 @@
           <t>Slovenia</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
       <c r="D79" t="n">
         <v>705</v>
       </c>
@@ -4611,17 +4083,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4639,7 +4105,6 @@
           <t>Somalia</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
         <v>706</v>
       </c>
@@ -4663,17 +4128,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4691,7 +4150,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="n">
         <v>710</v>
       </c>
@@ -4715,17 +4173,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4743,7 +4195,6 @@
           <t>Spain</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
         <v>724</v>
       </c>
@@ -4767,17 +4218,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4795,7 +4240,6 @@
           <t>Sri Lanka</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="n">
         <v>144</v>
       </c>
@@ -4819,17 +4263,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4847,7 +4285,6 @@
           <t>Sudan</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="n">
         <v>729</v>
       </c>
@@ -4871,17 +4308,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4899,7 +4330,6 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="n">
         <v>752</v>
       </c>
@@ -4923,17 +4353,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -4951,7 +4375,6 @@
           <t>Tanzania, United Republic of</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="n">
         <v>834</v>
       </c>
@@ -4975,17 +4398,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5003,7 +4420,6 @@
           <t>Thailand</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="n">
         <v>764</v>
       </c>
@@ -5027,17 +4443,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5055,7 +4465,6 @@
           <t>Timor-Leste</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
         <v>626</v>
       </c>
@@ -5079,17 +4488,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5107,7 +4510,6 @@
           <t>Trinidad and Tobago</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
         <v>780</v>
       </c>
@@ -5131,17 +4533,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5159,7 +4555,6 @@
           <t>Turkmenistan</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="n">
         <v>795</v>
       </c>
@@ -5183,17 +4578,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5211,7 +4600,6 @@
           <t>Türkiye</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
         <v>792</v>
       </c>
@@ -5235,17 +4623,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5263,7 +4645,6 @@
           <t>Uganda</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="n">
         <v>800</v>
       </c>
@@ -5287,17 +4668,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5315,7 +4690,6 @@
           <t>Ukraine</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="n">
         <v>804</v>
       </c>
@@ -5339,17 +4713,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5367,7 +4735,6 @@
           <t>United Arab Emirates</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="n">
         <v>784</v>
       </c>
@@ -5391,17 +4758,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5419,7 +4780,6 @@
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="n">
         <v>826</v>
       </c>
@@ -5443,17 +4803,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5471,7 +4825,6 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
         <v>840</v>
       </c>
@@ -5495,17 +4848,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5523,7 +4870,6 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
         <v>858</v>
       </c>
@@ -5547,17 +4893,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5575,7 +4915,6 @@
           <t>Uzbekistan</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="n">
         <v>860</v>
       </c>
@@ -5599,17 +4938,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5627,7 +4960,6 @@
           <t>Viet Nam</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
         <v>704</v>
       </c>
@@ -5651,17 +4983,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5679,7 +5005,6 @@
           <t>Zimbabwe</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="n">
         <v>716</v>
       </c>
@@ -5703,17 +5028,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr">
         <is>
           <t>auto-seeded from urls_deanscrape.txt</t>
@@ -5764,8 +5083,6 @@
           <t>Milei, Fernández, Macri, Kirchner</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>Spanish</t>
@@ -5836,8 +5153,6 @@
           <t>Macron</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>French</t>
@@ -5908,8 +5223,6 @@
           <t>Sheinbaum, López Obrador (paging back)</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>Spanish</t>
@@ -5933,6 +5246,81 @@
       <c r="P103" t="inlineStr">
         <is>
           <t>recipe: recipes/mex_presidencia.yml — validated live</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>chl_presidencia</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>South America</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>152</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>prensa.presidencia.cl</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>https://prensa.presidencia.cl/</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Bachelet, Piñera, Boric</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2014-03-11</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>recipe: recipes/chl_presidencia.yml</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Wayback-backed Argentina history
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -5100,12 +5100,12 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>recipe: recipes/arg_casarosada.yml — validated live</t>
+          <t>recipe: recipes/arg_casarosada.yml — Wayback-backed archive recipe</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Colombia presidency recipe
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P104"/>
+  <dimension ref="A1:P105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5324,6 +5324,71 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>col_presidencia</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>South America</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>170</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>presidencia.gov.co</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>https://www.presidencia.gov.co/prensa/Paginas/discursos.aspx</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Petro, Duque, Santos, Uribe</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>recipe: recipes/col_presidencia.yml — pending probe</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove curated source regeneration
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P105"/>
+  <dimension ref="A1:P104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5324,71 +5324,6 @@
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>col_presidencia</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>South America</t>
-        </is>
-      </c>
-      <c r="D105" t="n">
-        <v>170</v>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>presidencia.gov.co</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>https://www.presidencia.gov.co/prensa/Paginas/discursos.aspx</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>official_gov</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>static</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>Petro, Duque, Santos, Uribe</t>
-        </is>
-      </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>Spanish</t>
-        </is>
-      </c>
-      <c r="M105" t="inlineStr">
-        <is>
-          <t>fulltext</t>
-        </is>
-      </c>
-      <c r="N105" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="P105" t="inlineStr">
-        <is>
-          <t>recipe: recipes/col_presidencia.yml — pending probe</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Ireland recipe pagination
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2584,21 +2581,13 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>static</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>English</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>validated</t>
-        </is>
-      </c>
-      <c r="O46" s="1" t="n">
-        <v>46202</v>
+          <t>none</t>
+        </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
cleaning, curating, metadata scripts -- creating issues prepared
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -2586,7 +2586,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>validated</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>validated</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">

</xml_diff>

<commit_message>
master_sources.xlsx: fix mys_pmo source_url
/ucapan/ is a dead legacy ex-PM archive (stops ~2020); the live current-PM
source is the EN WordPress category /en/category/speeches-en/ (matches
recipes/mys_pmo.yml). Note appended to the row.

Follow-on to 869b47f (kept as a separate commit rather than an amend, since
869b47f was already pushed).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -6294,7 +6294,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>https://www.pmo.gov.my/ucapan/</t>
+          <t>https://www.pmo.gov.my/en/category/speeches-en/</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -6333,9 +6333,14 @@
           <t>draft</t>
         </is>
       </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>PM's Office 'ucapan' (speeches) section (base verified). Backlog target.</t>
+          <t>PM's Office 'ucapan' (speeches) section (base verified). Backlog target. || [2026-07-09] source_url fixed: /ucapan/ is a dead legacy archive of ex-PMs (stops ~2020); the live current-PM source is the EN WordPress category /en/category/speeches-en/ (382 links, 2024-2026, Anwar). Recipe recipes/mys_pmo.yml.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dynamic web crawling + a few more recipes
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q158"/>
+  <dimension ref="A1:Q166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>http://www.presidencymaldives.gov.mv/</t>
+          <t>https://presidency.gov.mv/Press/Articles/12</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3417,12 +3417,42 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Gayoom; Nasheed; Waheed; Yameen; Solih; Muizzu</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>1979</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>English</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>SOLVED - correction to earlier 'CF-blocked SPA'. The master's www.presidencymaldives.gov.mv is a Cloudflare-gated redirect whose DESTINATION, presidency.gov.mv, is a PLAIN STATIC site with no CF - target it directly. Probe-validated GREEN: 474 speeches 1979-2026, text .article-body + date .small-text. Speeches = category /Press/Articles/12, ?page=N pager (~48 pages); articles /Press/Article/&lt;id&gt;; date is .small-text under the h1 (NOT .date-text = recent-releases sidebar). Speaker via tenure crosscheck (6 presidents). Recipe: recipes/mdv_presidencymaldives.yml. FULL RUN pending.</t>
         </is>
       </c>
     </row>
@@ -3457,12 +3487,32 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>cdp</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>2026</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>SOLVED via renderer: cdp (engine issue #62, now implemented). LIVE Malta Presidency. Cloudflare bot-management fingerprint-blocks Playwright's own Chromium (headless AND headful) on detail pages; attaching over CDP to a user-launched real Chrome clears it. Probe-validated GREEN via CDP: 18 links, title h1.elementor-heading-title + text .elementor-widget-theme-post-content + date from the Elementor listing card (item_date, 'Month D, YYYY') all green. WordPress+Elementor; /speeches/&lt;slug&gt; + /speeches/N/ pager. TO RUN: launch Chrome with --remote-debugging-port=9222 (see docs/recipes.md 'Cloudflare-blocked sites'), then scrape; endpoint defaults to localhost:9222. Browser-free fallback for history: mlt_president_wayback (519 speeches). Speaker via tenure crosscheck. Recipe: recipes/mlt_president.yml.</t>
         </is>
       </c>
     </row>
@@ -3505,6 +3555,16 @@
           <t>none</t>
         </is>
       </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Broad gob.mx root - superseded for presidential speeches by mex_presidencia (gob.mx/presidencia, validated) + mex_presidencia_wayback (AMLO). Left as-is; no separate recipe needed.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3537,12 +3597,37 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Romanian</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Probe-validated: 202+ speeches 2013-2026 (Sandu/Dodon/Timofti), text &lt;article&gt;, date &lt;time datetime&gt;. Static, broken TLS -&gt; verify_ssl:false. Per-year CakePHP listings /rom/discursuri/index/YYYY/page:N via path pagination; individual speeches /rom/discursuri/&lt;slug&gt;. Added a politeness block (site throttles ~50 rapid requests -&gt; WinError 10060); keep pacing on FULL RUN. Speaker via tenure crosscheck (3 presidents). Original language Romanian (/eng mirror not used). Recipe: recipes/mda_presedinte.yml. FULL RUN pending.</t>
         </is>
       </c>
     </row>
@@ -3577,12 +3662,27 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Recipe recipes/mar_diplomatie.yml SHIPPED. Arabic ORIGINAL of the King's speeches (complements maroc.ma's English - see new mar_maroc row). Static Drupal; F5/BIG-IP ASM UA-keyed WAF -&gt; browser user_agent; broken TLS -&gt; verify_ssl:false. Scraping WORKS (title h1 + text .field--name-body, 5-7k chars). Two non-blocking caveats: (1) dates are Maghrebi Arabic month names (نونبر/يوليوز/غشت) that dateparser cannot read -&gt; left blank for the cleaner's corrected-date pass (speaker_default King Mohammed VI keeps the tenure crosscheck valid; a Maghrebi-month engine map would fix it at scrape time - see engine issue); (2) probe harvested ~14 links, pagination may be shallow/AJAX beyond page 0 - confirm depth on FULL RUN.</t>
         </is>
       </c>
     </row>
@@ -3617,12 +3717,32 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>2026</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Recipe recipes/nld_royalhouse.yml (NB source_id spelling differs from this row's 'nld_royal-house' - reconcile). King Willem-Alexander + royals. Platform-Rijksoverheid Search-UI SPA -&gt; renderer:js; cursor pager not chainable, so the ~60 cursor pages ?current=n_&lt;page&gt;_n are enumerated as 64 start_urls (type:none). Detail pages static (text &lt;main&gt;), date from the /documents/YYYY/MM/DD/ URL. ~600 docs to 2004; cleaner keeps the reigning head of state. Head-of-government companion nld_rijksoverheid is blocked (see its row). Probe-green.</t>
         </is>
       </c>
     </row>
@@ -3657,12 +3777,27 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>cdp</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>2026</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>SOLVED via renderer: cdp (engine issue #62). New Zealand Governor-General, gg.govt.nz. Cloudflare 'Just a moment' CRASHES the engine's headless Chromium (Page.goto: Page crashed); a user-launched real Chrome via CDP clears it. Probe-validated GREEN via CDP: 60 links, title h1 + text &lt;main&gt; + date &lt;time datetime&gt; all green. Listing /publications/&lt;slug&gt; + 0-indexed ?page= pager. TO RUN: launch Chrome with --remote-debugging-port=9222 (see docs/recipes.md), then scrape. NZ head of government is separately covered green by nzl_beehive. FULL RUN confirms the archive floor. Recipe: recipes/nzl_gg.yml.</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3844,17 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Google Books entry (Obasanjo) - not scrapable as a config recipe. Obasanjo-era speeches would need a different source/approach. The working Nigeria sources are nga_statehouse (live, Tinubu+Buhari 2019-) and nga_statehouse_wayback (Buhari first term 2015-2019).</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3891,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>static</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3754,9 +3899,29 @@
           <t>Bola Ahmed Tinubu</t>
         </is>
       </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="N69" t="inlineStr">
         <is>
           <t>draft</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Re-validated (spread green: text .news-detail-content, date .page-info; 272 links 2019-2026 across Tinubu/Buhari/Osinbajo). Live archive floor ~2019-04 (site rebuilt then). Buhari FIRST term 2015-2019 is covered by the NEW nga_statehouse_wayback companion. Speaker cleaner-assigned. FULL RUN pending.</t>
         </is>
       </c>
     </row>
@@ -3791,12 +3956,37 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Macedonian</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Probe-validated (12/12 spread): 123 items 2024-05..2026-07, all fields green. WordPress (Divi) via WP REST API /wp-json/wp/v2/posts (Macedonian speech cats 5 obrakjanja + 3 intervjua; EN/Albanian dup cats excluded); body .et_pb_post_content. Cloudflare non-challenging to the bot UA. Speaker Siljanovska-Davkova. Predecessor Pendarovski (2019-2024) is NOT in the live WP and looks thin in Wayback (mostly listing pages) - possible follow-up. FULL RUN pending.</t>
         </is>
       </c>
     </row>
@@ -3831,12 +4021,37 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Norwegian</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Probe-validated (10/10 spread): 1232 sitemap speeches (fra_elysee pattern), sampled 2013-2025, archive reaches ~2005. King Harald V + Queen Sonja + Crown Prince Haakon + Crown Princess Mette-Marit. SSR site (Vercel), bot-UA OK. No &lt;time&gt; -&gt; date regex from the Norwegian header line (date_languages nb); speaker from the URL /taler-og-budskap/&lt;royal&gt;/ slug (cleaner normalises, tenure crosscheck keeps head of state). royalcourt.no is the English mirror (not used). Head-of-government companion nor_regjeringen is blocked (see its row). FULL RUN pending.</t>
         </is>
       </c>
     </row>
@@ -5233,6 +5448,16 @@
           <t>Sheinbaum, López Obrador (paging back)</t>
         </is>
       </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="L104" t="inlineStr">
         <is>
           <t>Spanish</t>
@@ -5250,12 +5475,12 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>recipe: recipes/mex_presidencia.yml — validated live</t>
+          <t>Re-validated (spread green: text .article-body, date, context). CHANGE: raised max_pages 50-&gt;130. The filter_origin=archive listing covers ONLY the CURRENT presidency (Sheinbaum, from 2024-10): page ~105 = 2024-10-23, page ~200 empty. max_pages 50 truncated it at ~2025-09 (~11 of ~22 months); 130 captures her full term. AMLO 2018-2024 is NOT in this archive -&gt; NEW mex_presidencia_wayback companion. Speaker cleaner-assigned. FULL RUN pending.</t>
         </is>
       </c>
     </row>
@@ -8906,6 +9131,616 @@
       <c r="Q158" t="inlineStr">
         <is>
           <t>Live presidence.gov.mg is broken (nginx-404) -&gt; wayback. recipes/mdg_presidence_wayback.yml probe-validated for TITLE+TEXT: 1745 Joomla /actualites items 2014-2026. DATE PARTIAL (no clean date element; in-text French regex; relies on downstream date-correction). FULL RUN pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>mar_maroc</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>504</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>maroc.ma (Royal Speeches, EN)</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>https://maroc.ma/en/royal-speeches-and-messages/royal-speeches</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>King Mohammed VI</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>NEW SOURCE (canonical royal portal; the master's mar_diplomatie is the second, Arabic, source). Probe-validated (10/10 spread): 60 speeches 2012-07..2025-10, all fields green. Official ENGLISH translation. Static Drupal, bot-UA OK. Body .c-wysiwyg; date from the listing card .item-time (DD-MM-YYYY, day-first via 'fr') because the article page's only &lt;time&gt; is a related-news sidebar. 0-indexed Drupal pager (start:0). COVERAGE GAP: floor 2012 (Mohammed VI reigns since 1999); 1999-2012 hard to source. Recipe: recipes/mar_maroc.yml. FULL RUN pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>mex_presidencia_wayback</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>484</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>gob.mx/presidencia (Wayback, AMLO)</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/2/https://www.gob.mx/presidencia/articulos/version-estenografica</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Andres Manuel Lopez Obrador</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>2018-12</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>NEW - Wayback companion to mex_presidencia for the AMLO era (absent from the live archive). Probe-validated: 3475 CDX snapshots, text .article-body 4k-65k chars, date, context green. Two CDX prefixes for the mid-term URL-path change. wayback_to 20241001 hands off to the live recipe. High volume (~2000+ daily transcripts). Recipe: recipes/mex_presidencia_wayback.yml. FULL RUN pending (heavy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>nzl_beehive</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>554</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>beehive.govt.nz (Speeches)</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>https://www.beehive.govt.nz/speeches</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>NZ Prime Minister + ministers</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>NEW - head-of-government companion to the listed Governor-General source nzl_gg. Probe-validated (spread green over 3-page subset: title h1, text &lt;main&gt; 9k-21k chars, date &lt;time&gt;). Imperva Incapsula JS challenge cleared by renderer:js (httpx gets a 212-byte _Incapsula_Resource stub). Listing /speech/&lt;slug&gt; + 0-indexed ?page= pager; archive to mid/late-2000s (max_pages 200, auto-stops). All-of-government - cleaner keeps the PM's. Recipe: recipes/nzl_beehive.yml. FULL RUN pending (js render of ~100+ pages).</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>nor_regjeringen</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>578</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>regjeringen.no (Taler og innlegg)</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>https://www.regjeringen.no/no/aktuelt/taler_artikler/id1334/</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Norwegian PM + ministers</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Norwegian</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>NEW - head-of-government source (companion to nor_kongehuset). BLOCKED here: Cloudflare 'Just a moment' on ALL HTML (listing + detail, both UAs -&gt; 403), and headless Chromium did NOT clear it even after 9s (harder than gg.govt.nz, which clears at ~7s). The RSS feed /&lt;lang&gt;/rss/Rss/1334/ bypasses CF but is summary-only (~45 items, 118-char descriptions, no pagination) and its links go to CF-blocked detail pages. FIX: (1) run from a residential IP (may clear the challenge); (2) Wayback of /no/aktuelt/&lt;slug&gt;/id&lt;N&gt;/ (server-rendered full text, but /aktuelt/ mixes all doc types - large noisy crawl needing the cleaner's gate). Norway's head of state (King) is covered green by nor_kongehuset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>nld_rijksoverheid</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>528</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>rijksoverheid.nl (toespraken)</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>https://www.rijksoverheid.nl/documenten?type=toespraak</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Dutch PM + ministers</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>NEW - head-of-government source (companion to nld_royalhouse). Detail pages ARE static (full text in &lt;main&gt;; date in the /documenten/YYYY/MM/DD/ URL). BLOCKER is the LISTING: a JS Search-UI SPA, no sitemap (sitemaps are nav-only), no RSS. renderer:js renders results but ?type=toespraak is NOT applied on direct load (header 'Alle documenten'; results mix in non-speeches) and pagination is a hash-signed POST /api/search the engine cannot drive, plus a cursor ?current=n_N (drops the type param). FIX: find the correct filtered feed/endpoint, then renderer:js + scoped result list + text &lt;main&gt; + date url_regex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>nga_statehouse_wayback</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>566</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>statehouse.gov.ng (Wayback, old Joomla)</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/2/http://www.statehouse.gov.ng/index.php/news</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Muhammadu Buhari (2015-2019)</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>NEW - Wayback companion to nga_statehouse for Buhari's FIRST term. Probe-validated on scraping: 705 snapshots, title .item-page h2 + text .item-page green (1k-9k chars). Old Joomla /index.php/news/&lt;id&gt;-&lt;slug&gt;. ONLY gap is date: the old pages carry NO date element/in-body date, so date is left blank for the cleaner's corrected-date pass (speaker_default Buhari keeps the tenure crosscheck valid). Engine follow-up: use the Wayback capture timestamp as a date fallback. Recipe: recipes/nga_statehouse_wayback.yml. FULL RUN pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>mlt_president_wayback</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Malta</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>470</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>president.gov.mt (Wayback)</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/2/https://president.gov.mt/diskors</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>George Vella (2019-2024); earlier presidents; early Spiteri Debono</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>NEW - Wayback recipe for the CF-blocked president.gov.mt (probe-green fallback for the live mlt_president). Probe-validated: 519 snapshots, text .elementor-widget-theme-post-content 2.7k-25k chars, date .elementor-post-info__item--type-date (DD.MM.YYYY day-first via 'fr'). WordPress+Elementor; ~985 archived speech pages across redesigns (/diskors-&lt;slug&gt;, /speeches/&lt;slug&gt;, /the-presidents-address-&lt;slug&gt;). A few newer /speeches/ pages lack the date widget. Bilingual EN+MT. Recipe: recipes/mlt_president_wayback.yml. FULL RUN pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>mlt_gov</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Malta</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>470</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>gov.mt / opm.gov.mt (Malta Government / OPM)</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>https://www.gov.mt/</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>official_gov</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Malta Prime Minister (Robert Abela)</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>fulltext</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>NEW - head-of-government source (companion to the listed president source). BLOCKED from this environment, but likely works in a normal browser (same Cloudflare bot-management as president.gov.mt, which the researcher confirmed reads fine on a residential IP). gov.mt, opm.gov.mt (Office of the PM), doi.gov.mt (also broken TLS) and parlament.mt all returned CF 'Attention Required' to httpx from this datacenter IP. I could NOT locate a clean PM 'speeches' listing before the block. FIX: from a residential IP, find the OPM/DOI speeches listing URL, then a renderer:js recipe (or Wayback of it). Not a firewall - bot-management + datacenter-IP fingerprint.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remaining wayback recipes N-Z
</commit_message>
<xml_diff>
--- a/data/sources/master_sources.xlsx
+++ b/data/sources/master_sources.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="1279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="1383">
   <si>
     <t>source_id</t>
   </si>
@@ -3854,6 +3854,318 @@
   </si>
   <si>
     <t xml:space="preserve">Probe-validated 2026-07-26 (--spread --n 8): 4,252 date-path post captures (president.go.ke/&lt;yyyy&gt;/&lt;mm&gt;/&lt;dd&gt;/&lt;slug&gt;/, CDX prefix president.go.ke/20 ~8,000 raw). The OLD pre-Elementor WordPress site (Uhuru Kenyatta era, president 2013-2022) archives as CLEAN HTML (unlike the modern Elementor /speeches_remarks/ JS shells). TITLE(h1.entry-title) clean; TEXT via .entry-content/generic fallback (2.7k-3.9k chars); DATE from the URL permalink via url_regex ONLY (unambiguous ISO; .post-date returns a re-crawl artifact). Posts mix speeches + presidency news -&gt; cleaner document-type gate keeps the speech/official_statement subset. NO speaker_default (Uhuru + First Lady Margaret Kenyatta + quoted ministers) -&gt; cleaner speaker pass + tenure crosscheck. 'yes-and' to the live ken_president (Ruto 2022- PDFs): this is the Kenyatta 2013-2022 corpus. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can_pmo_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Minister's Office pm.gc.ca speeches (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://pm.gc.ca/en/news/speeches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Justin Trudeau; Mark Carney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 417 dated /en/news/speeches/&lt;yyyy&gt;/&lt;mm&gt;/&lt;dd&gt;/&lt;slug&gt; snapshots. TEXT(.field--name-body) 4.2k-16k chars + DATE(url_regex from the permalink) 2015-2026 all green (Trudeau + Carney). TITLE from the URL slug via url_regex (the archived Drupal h1 is a nav blob, and selectors win over url_regex, so title uses url_regex ONLY) -&gt; cleaner polishes dashes. OVERLAP: ~1,000 Canada Dean_scrape speeches (2000-2022) already exist -&gt; additive value is mainly the 2022-&gt; tail + PM Carney (2025- ) + snapshot-insurance; the merge dedupes. Old /eng/news Harper-era scheme (~90% Drupal asset junk, likely inside Dean_scrape) NOT harvested. NO speaker_default. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">idn_setkab_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indonesia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabinet Secretariat setkab.go.id/en transcripts (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://setkab.go.id/en/category/speech-transcript/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joko Widodo; Prabowo Subianto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 1,964 snapshots. The transcript-slug link_pattern (remarks/statement/press-statement/address/... of the President) cleanly ISOLATES the president's English transcripts from the aggregator's general /en/ news -&gt; every sample is a genuine transcript (Jokowi/Prabowo: 'Address of President... at Georgetown University'; 'Press Statement of President...'; 'Remarks of President...'). TITLE(h1) + TEXT(.detail_text, 1.9k-37k chars) + DATE(meta article:published_time) all green (2021-2025; one older page falls to the cleaner). English -&gt; English column, no MT. 'yes-and' companion to the live idn_setkab (recovers older/deleted transcripts). NO verify_ssl needed (fetch is from the Archive). NO speaker_default. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ind_pmindia_nic_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">356</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Old PMO pmindia.nic.in speeches (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://pmindia.nic.in/speech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manmohan Singh; Atal Bihari Vajpayee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 1,185 snapshots. NEW pre-Modi historical depth: the OLD pmindia.nic.in holds full English speeches of PM Manmohan Singh (2004-2014) via /speech/content.asp?id=&lt;id&gt; -&gt; TEXT(td) 25k-48k chars, DATE(body dateline) 2004-2011 all green (TITLE is the generic 'Prime Minister's Office' banner -&gt; the cleaner derives a title from the body, the aus_gg pattern). The /speech-details.php?nodeid= PHP tail (2012-2014) extracts thinly (generic backstop). NO speaker_default (Vajpayee ...2004 + Manmohan Singh 2004-2014) -&gt; cleaner + tenure crosscheck. Nothing else in the corpus covers pre-Modi Indian PMs. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ind_pmindia_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM of India pmindia.gov.in/en/news_updates (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pmindia.gov.in/en/news_updates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Narendra Modi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 15,926 /en/news_updates snapshots. TITLE(.content-block h2 — the bare h1 is the site logo) + TEXT(.news-bg, up to 28.8k chars) + DATE(.date) all green; speaker_default Narendra Modi (2014-2026). WAF WORK-AROUND: pmindia.gov.in's UA-keyed WAF blocks the live bot UA, but the Archive serves the pages cleanly (no user_agent needed). 'yes-and' companion to the live ind_pmindia. Detail pages mix PM speeches/statements + short press notes -&gt; document_type gate filters. Companion ind_pmindia_nic_wayback covers the pre-Modi PMs. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kaz_akorda_english_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kazakhstan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">akorda.kz English state-of-nation addresses (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://akorda.kz/en/addresses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nursultan Nazarbayev; Kassym-Jomart Tokayev</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): the /en/addresses/addresses_of_president/&lt;slug&gt; article extracts cleanly -&gt; TITLE(h1) 'State of the Nation Address', TEXT(.text) 34,036 chars, DATE(.date) 2017-01-31. NARROWED to /en/addresses/ (CDX approx 46 caps 2015-2024) -- the annual state-of-the-nation Addresses of Presidents Nazarbayev + Tokayev, the highest-value single speeches. ENGLISH sibling of the native (Russian) kaz_akorda_wayback -&gt; English column, no MT. The broader /en/speeches/&lt;cat&gt;/&lt;slug&gt; tree (approx 314 caps) archives its OLDER captures as shells/section-listings (.text -&gt; 0; generic ~0.8-2k of chrome) -&gt; DEFERRED as a follow-up (that content is covered by the native Russian recipe + translation). NO speaker_default. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mar_maroc_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morocco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maroc.ma royal speeches EN (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maroc.ma/en/royal-speeches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">King Mohammed VI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 178 snapshots. GENUINE English -&gt; TITLE(h1) clean ('Full Speech of HM the King on COP22 High-Level Segment'; 'Full Text of Royal Message to the 27th African Union Summit'); NEW scheme body via .c-wysiwyg (7918 chars), OLD /en/royal-speeches/&lt;slug&gt; scheme (2013-2024) body via the engine's generic fallback (5.8k-13k chars). DATE deferred to cleaner + wayback_capture (the article's only &lt;time&gt; is a related-news sidebar). speaker_default King Mohammed VI. Official English translation -&gt; English column, no MT. 'yes-and' companion to the live mar_maroc (current scheme); recovers the relocated OLD-scheme royal speeches. Companion Arabic original is mar_diplomatie. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mdv_presidencymaldives_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maldives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">462</t>
+  </si>
+  <si>
+    <t xml:space="preserve">President's Office presidency.gov.mv (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://presidency.gov.mv/Press/Article/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maumoon Abdul Gayoom; Mohamed Nasheed; Mohammed Waheed; Abdulla Yameen; Ibrahim Mohamed Solih; Mohamed Muizzu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 35,300 /Press/Article/&lt;id&gt; snapshots. TITLE(h1) + TEXT(.article-body, 614-2985 chars) green; DATE(.small-text) parses English dates (2011-05-29 Nasheed, 2018-08-20, 2023-10-16) and falls to the cleaner for Dhivehi-month dates. 'yes-and' companion to the live mdv_presidencymaldives (which paginates /Press/Articles/12 back to ~1979): a frozen snapshot + deleted-article insurance for the same current DB. Mixed English/Dhivehi (cleaner detects per-doc). NO speaker_default. The much older presidencymaldives.gov.mv ASP/PHP generation is NOT harvested (messy multi-scheme lead). FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sgp_pmo_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Singapore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">702</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Minister's Office pmo.gov.sg (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pmo.gov.sg/newsroom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lee Hsien Loong; Heng Swee Keat; Teo Chee Hean; Lawrence Wong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 3,269 /Newsroom snapshots. The OLDER /Newsroom/&lt;Title-Case-slug&gt; CMS generation archives with REAL bodies (NOT JS shells): TITLE(h1) clean ('PM Lee Hsien Loong at the DSO50 Jubilee Dinner'; 'Eulogy by PM Lee Hsien Loong at funeral of the late Mr S R Nathan'), TEXT(article/main, 5.9k-11.9k chars), DATE(article regex) 2011-2026 all green. Covers PM Lee Hsien Loong / DPM Heng Swee Keat / DPM Teo Chee Hean (pre-2024). 'yes-and' companion to the live sgp_pmo (current Isomer sitemap). NO speaker_default. Distinct from the ceremonial-President sgp_istana / sgp_istana_wayback. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sle_statehouse_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sierra Leone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">694</t>
+  </si>
+  <si>
+    <t xml:space="preserve">State House statehouse.gov.sl date-path posts (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://statehouse.gov.sl/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Julius Maada Bio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 280 date-path /YYYY/MM/DD/&lt;slug&gt; snapshots. TITLE(h1) + TEXT(.elementor-widget-theme-post-content, 1.3k-4k chars for substantive posts; some 43-101-char stubs) + DATE(url_regex) green (President Julius Maada Bio). CAVEAT: the archived SLUGGED posts are almost all 2025-2026 — the pre-2025 era was captured only as bare /YYYY/MM/DD/ day-listings, so the hoped 2018-2024 Bio depth is NOT recoverable via wayback -&gt; this largely OVERLAPS the live sle_statehouse (WP REST, 2025-01+); value = frozen snapshot + deleted-post insurance. NO speaker_default (Bio + a brief late-Koroma window) -&gt; cleaner + tenure. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">syc_statehouse_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seychelles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">690</t>
+  </si>
+  <si>
+    <t xml:space="preserve">State House statehouse.gov.sc/speeches (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.statehouse.gov.sc/speeches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">James Michel; Danny Faure; Wavel Ramkalawan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 841 /speeches/&lt;id&gt;/&lt;slug&gt; snapshots. TITLE(h1) clean speech titles for the OLD-layout majority (Michel/Faure era); TEXT(.container/.u-sheet-1, 3.4k-9.4k chars) green; DATE mostly falls to the cleaner (old captures lack the modern Nicepage p.u-text-2 date element; wayback_capture backstops). Spans President James Michel (2004-2016), Danny Faure (2016-2020), Wavel Ramkalawan (2020- ) + VP remarks. Multilingual site: default /speeches is English but some captures are the French/Creole version (cleaner detects per-doc). 'yes-and' companion to the live syc_statehouse. NO speaker_default. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tto_otp_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trinidad and Tobago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">780</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office of the President otp.tt (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://otp.tt/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paula-Mae Weekes; Christine Kangaloo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 845 single-segment WordPress-post snapshots. TITLE(h1.entry-title) clean ('Christmas Message from Her Excellency'; 'Message for the International Day of Education'; 'President Weekes participates in Walk for Sight 2019'); TEXT(.entry-content, 505-3058 chars) green. DATE: the archived Elementor pages expose no clean date element -&gt; date falls to the cleaner's corrected-date pass + wayback_capture. GREENFIELD (Office of the President; T&amp;T's ceremonial head of state - Presidents Paula-Mae Weekes 2018-2023, Christine Kangaloo 2023- ). Mostly ceremonial notices (appointments, courtesy calls) + genuine messages/speeches -&gt; the document_type gate keeps the substantive addresses. NO speaker_default. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uga_statehouse_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uganda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">State House statehouse.go.ug/media/speeches (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://statehouse.go.ug/media/speeches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yoweri Museveni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 127 dated /media/speeches/&lt;yyyy&gt;/&lt;mm&gt;/&lt;dd&gt;/&lt;slug&gt; snapshots. TITLE(h1) clean ('State of the Nation Address 2013'; 'President Museveni''s 54th Independence Day Speech'); TEXT(.content, 16k-46k chars - full addresses) + DATE(url_regex from the permalink) 2011-2022 all green. GREENFIELD (President Yoweri Museveni, in office since 1986). The link_pattern keeps /media/speeches/&lt;date&gt;/&lt;slug&gt; articles and drops the 2021 crawl-storm of ?page=N day-listings. NO speaker_default (Museveni dominant + occasional VP/official remarks) -&gt; cleaner + tenure crosscheck. The 2023+ site uses a different flat-slug scheme (not covered here). FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaf_gov_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Africa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">710</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SA Government speeches gov.za/news/speeches (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.gov.za/news/speeches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyril Ramaphosa; Jacob Zuma; + ministers/premiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 14,886 /news/speeches snapshots. TITLE(h1) + TEXT(.field--name-body, 4.4k-42k chars) + DATE(&lt;time&gt;) all green, content back to 2009 (UKZN 2009; Madonsela 2010) through 2025. Deep official aggregator of ALL SA government speeches (President Ramaphosa + ministers + premiers + Speaker). 'yes-and' companion to the live zaf_gov (frozen snapshot + deleted-article insurance of the same migrated DB). Distinct from zaf_thepresidency_wayback (the presidency's own old Drupal-7 site). NO speaker_default -&gt; the cleaner's speaker pass keeps the President's speeches + document_type gate filters ministers. FULL RUN is the researcher's gate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zwe_theopc_wayback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zimbabwe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office of the President and Cabinet theopc.gov.zw (Wayback/CDX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://www.theopc.gov.zw/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emmerson Mnangagwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe-validated 2026-07-27 (--spread --n 8): 177 Joomla /index.php/&lt;id&gt;-&lt;slug&gt; snapshots. TEXT(article) 217-46,185 chars (transcript of President ED's Financial Times interview 46k; Independence Day speech 22k) + DATE(.published) 2016-2020 all green. TITLE is 'Latest News' (chrome) on the bare news items -&gt; the cleaner derives a title from the body; the /index.php/news/speeches-and-statements/ category page carries a real h1. GREENFIELD (Zimbabwe OPC; President Emmerson Mnangagwa 2017- , 'Second Republic'). NO speaker_default (Mnangagwa dominant + occasional chief-secretary statements) -&gt; cleaner + document_type gate. FULL RUN is the researcher's gate.</t>
   </si>
 </sst>
 </file>
@@ -12966,6 +13278,748 @@
         <v>1279</v>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B217" t="s">
+        <v>1281</v>
+      </c>
+      <c r="C217" t="s">
+        <v>1265</v>
+      </c>
+      <c r="D217" t="s">
+        <v>1282</v>
+      </c>
+      <c r="E217" t="s">
+        <v>1283</v>
+      </c>
+      <c r="F217" t="s">
+        <v>1284</v>
+      </c>
+      <c r="G217" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H217" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I217" t="s">
+        <v>1285</v>
+      </c>
+      <c r="J217" t="s">
+        <v>1243</v>
+      </c>
+      <c r="K217" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L217" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M217" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N217" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O217" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P217" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q217" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B218" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C218" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D218" t="s">
+        <v>1290</v>
+      </c>
+      <c r="E218" t="s">
+        <v>1291</v>
+      </c>
+      <c r="F218" t="s">
+        <v>1292</v>
+      </c>
+      <c r="G218" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H218" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I218" t="s">
+        <v>1293</v>
+      </c>
+      <c r="J218" t="s">
+        <v>1243</v>
+      </c>
+      <c r="K218" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L218" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M218" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N218" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O218" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P218" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q218" t="s">
+        <v>1294</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="s">
+        <v>1295</v>
+      </c>
+      <c r="B219" t="s">
+        <v>1296</v>
+      </c>
+      <c r="C219" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D219" t="s">
+        <v>1297</v>
+      </c>
+      <c r="E219" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F219" t="s">
+        <v>1299</v>
+      </c>
+      <c r="G219" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H219" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I219" t="s">
+        <v>1300</v>
+      </c>
+      <c r="J219" t="s">
+        <v>1301</v>
+      </c>
+      <c r="K219" t="s">
+        <v>1278</v>
+      </c>
+      <c r="L219" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M219" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N219" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O219" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P219" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q219" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B220" t="s">
+        <v>1296</v>
+      </c>
+      <c r="C220" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D220" t="s">
+        <v>1297</v>
+      </c>
+      <c r="E220" t="s">
+        <v>1304</v>
+      </c>
+      <c r="F220" t="s">
+        <v>1305</v>
+      </c>
+      <c r="G220" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H220" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I220" t="s">
+        <v>1306</v>
+      </c>
+      <c r="J220" t="s">
+        <v>1278</v>
+      </c>
+      <c r="K220" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L220" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M220" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N220" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O220" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P220" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q220" t="s">
+        <v>1307</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B221" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C221" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D221" t="s">
+        <v>1310</v>
+      </c>
+      <c r="E221" t="s">
+        <v>1311</v>
+      </c>
+      <c r="F221" t="s">
+        <v>1312</v>
+      </c>
+      <c r="G221" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H221" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I221" t="s">
+        <v>1313</v>
+      </c>
+      <c r="J221" t="s">
+        <v>1243</v>
+      </c>
+      <c r="K221" t="s">
+        <v>1253</v>
+      </c>
+      <c r="L221" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M221" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N221" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O221" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P221" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q221" t="s">
+        <v>1314</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B222" t="s">
+        <v>1316</v>
+      </c>
+      <c r="C222" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D222" t="s">
+        <v>1317</v>
+      </c>
+      <c r="E222" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F222" t="s">
+        <v>1319</v>
+      </c>
+      <c r="G222" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H222" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I222" t="s">
+        <v>1320</v>
+      </c>
+      <c r="J222" t="s">
+        <v>1321</v>
+      </c>
+      <c r="K222" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L222" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M222" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N222" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O222" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P222" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q222" t="s">
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B223" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C223" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D223" t="s">
+        <v>1325</v>
+      </c>
+      <c r="E223" t="s">
+        <v>1326</v>
+      </c>
+      <c r="F223" t="s">
+        <v>1327</v>
+      </c>
+      <c r="G223" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H223" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I223" t="s">
+        <v>1328</v>
+      </c>
+      <c r="J223" t="s">
+        <v>1227</v>
+      </c>
+      <c r="K223" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L223" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M223" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N223" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O223" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P223" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q223" t="s">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B224" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C224" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D224" t="s">
+        <v>1332</v>
+      </c>
+      <c r="E224" t="s">
+        <v>1333</v>
+      </c>
+      <c r="F224" t="s">
+        <v>1334</v>
+      </c>
+      <c r="G224" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H224" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I224" t="s">
+        <v>1335</v>
+      </c>
+      <c r="J224" t="s">
+        <v>1242</v>
+      </c>
+      <c r="K224" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L224" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M224" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N224" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O224" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P224" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q224" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B225" t="s">
+        <v>1338</v>
+      </c>
+      <c r="C225" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D225" t="s">
+        <v>1339</v>
+      </c>
+      <c r="E225" t="s">
+        <v>1340</v>
+      </c>
+      <c r="F225" t="s">
+        <v>1341</v>
+      </c>
+      <c r="G225" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H225" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I225" t="s">
+        <v>1342</v>
+      </c>
+      <c r="J225" t="s">
+        <v>1343</v>
+      </c>
+      <c r="K225" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L225" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M225" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N225" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O225" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P225" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q225" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B226" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C226" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D226" t="s">
+        <v>1347</v>
+      </c>
+      <c r="E226" t="s">
+        <v>1348</v>
+      </c>
+      <c r="F226" t="s">
+        <v>1349</v>
+      </c>
+      <c r="G226" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H226" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I226" t="s">
+        <v>1350</v>
+      </c>
+      <c r="J226" t="s">
+        <v>1351</v>
+      </c>
+      <c r="K226" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L226" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M226" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N226" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O226" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P226" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q226" t="s">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="s">
+        <v>1353</v>
+      </c>
+      <c r="B227" t="s">
+        <v>1354</v>
+      </c>
+      <c r="C227" t="s">
+        <v>1265</v>
+      </c>
+      <c r="D227" t="s">
+        <v>1355</v>
+      </c>
+      <c r="E227" t="s">
+        <v>1356</v>
+      </c>
+      <c r="F227" t="s">
+        <v>1357</v>
+      </c>
+      <c r="G227" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H227" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I227" t="s">
+        <v>1358</v>
+      </c>
+      <c r="J227" t="s">
+        <v>1278</v>
+      </c>
+      <c r="K227" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L227" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M227" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N227" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O227" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P227" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q227" t="s">
+        <v>1359</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="s">
+        <v>1360</v>
+      </c>
+      <c r="B228" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C228" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D228" t="s">
+        <v>1362</v>
+      </c>
+      <c r="E228" t="s">
+        <v>1363</v>
+      </c>
+      <c r="F228" t="s">
+        <v>1364</v>
+      </c>
+      <c r="G228" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H228" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I228" t="s">
+        <v>1365</v>
+      </c>
+      <c r="J228" t="s">
+        <v>1242</v>
+      </c>
+      <c r="K228" t="s">
+        <v>1270</v>
+      </c>
+      <c r="L228" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M228" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N228" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O228" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P228" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q228" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B229" t="s">
+        <v>1368</v>
+      </c>
+      <c r="C229" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D229" t="s">
+        <v>1369</v>
+      </c>
+      <c r="E229" t="s">
+        <v>1370</v>
+      </c>
+      <c r="F229" t="s">
+        <v>1371</v>
+      </c>
+      <c r="G229" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H229" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I229" t="s">
+        <v>1372</v>
+      </c>
+      <c r="J229" t="s">
+        <v>1373</v>
+      </c>
+      <c r="K229" t="s">
+        <v>1228</v>
+      </c>
+      <c r="L229" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M229" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N229" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O229" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P229" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q229" t="s">
+        <v>1374</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B230" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C230" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D230" t="s">
+        <v>1377</v>
+      </c>
+      <c r="E230" t="s">
+        <v>1378</v>
+      </c>
+      <c r="F230" t="s">
+        <v>1379</v>
+      </c>
+      <c r="G230" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H230" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I230" t="s">
+        <v>1380</v>
+      </c>
+      <c r="J230" t="s">
+        <v>1381</v>
+      </c>
+      <c r="K230" t="s">
+        <v>1382</v>
+      </c>
+      <c r="L230" t="s">
+        <v>1229</v>
+      </c>
+      <c r="M230" t="s">
+        <v>1230</v>
+      </c>
+      <c r="N230" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O230" t="s">
+        <v>1232</v>
+      </c>
+      <c r="P230" t="s">
+        <v>1286</v>
+      </c>
+      <c r="Q230" t="s">
+        <v>1383</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0"/>

</xml_diff>